<commit_message>
hnaya dart slice time
</commit_message>
<xml_diff>
--- a/0B5F9D00.xlsx
+++ b/0B5F9D00.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\power bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{335AA08A-0D72-4D1E-B270-56EB7B506255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B859417-3B23-43F2-8931-D4E9E3C95B89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30BFA6B8-A676-4931-80C6-DA6F72E44419}"/>
   </bookViews>
@@ -20,12 +20,21 @@
   </sheets>
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="2" hidden="1">table!$A$1:$H$41</definedName>
+    <definedName name="NativeTimeline_Date">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="5" r:id="rId5"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}">
+      <x15:timelineCacheRefs>
+        <x15:timelineCacheRef r:id="rId6"/>
+      </x15:timelineCacheRefs>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -199,7 +208,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -209,12 +218,524 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="172" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="46">
+  <dxfs count="119">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -538,397 +1059,571 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>556260</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>18358</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>594360</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>141663</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="'data analysis'!A7">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="12" name="Group 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{298D81AF-3522-AE4E-1E11-5B9B0E9C0C11}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86F77C03-3584-0089-DE88-7E7005622D0B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2385060" y="701040"/>
-          <a:ext cx="1866900" cy="739140"/>
+          <a:off x="2438400" y="1664278"/>
+          <a:ext cx="1866900" cy="671945"/>
+          <a:chOff x="2385060" y="701040"/>
+          <a:chExt cx="1866900" cy="739140"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="'data analysis'!A7">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="2" name="TextBox 1">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{298D81AF-3522-AE4E-1E11-5B9B0E9C0C11}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2385060" y="701040"/>
+            <a:ext cx="1866900" cy="739140"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
           <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="95000"/>
             </a:schemeClr>
           </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:fld id="{E579ED93-EF0A-42B5-9B0D-24E1CFD28BCA}" type="TxLink">
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Aptos Narrow"/>
-            </a:rPr>
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr algn="r"/>
-            <a:t> $426,530 </a:t>
-          </a:fld>
-          <a:endParaRPr lang="en-US" sz="2000" b="1">
-            <a:latin typeface="Gotham" panose="02000504020000020004" pitchFamily="2" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+            <a:fld id="{E579ED93-EF0A-42B5-9B0D-24E1CFD28BCA}" type="TxLink">
+              <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Aptos Narrow"/>
+              </a:rPr>
+              <a:pPr algn="r"/>
+              <a:t> $290,180 </a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-US" sz="2000" b="1">
+              <a:latin typeface="Gotham" panose="02000504020000020004" pitchFamily="2" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="6" name="Graphic 5" descr="Money with solid fill">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAD87EE3-6A2A-DAE4-1F6A-4CBB4C810A49}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+            <a:extLst>
+              <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2522220" y="838200"/>
+            <a:ext cx="457200" cy="457200"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>240030</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>293370</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>18358</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>278130</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:colOff>331470</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>141663</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="'data analysis'!C7">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="TextBox 2">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="13" name="Group 12">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E128FE5D-66DC-2A53-2918-C5B556CBB598}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C648A276-A127-552E-5911-9F55C081F05D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5116830" y="701040"/>
-          <a:ext cx="1866900" cy="739140"/>
+          <a:off x="5170170" y="1664278"/>
+          <a:ext cx="1866900" cy="671945"/>
+          <a:chOff x="5116830" y="701040"/>
+          <a:chExt cx="1866900" cy="739140"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="'data analysis'!C7">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="3" name="TextBox 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E128FE5D-66DC-2A53-2918-C5B556CBB598}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5116830" y="701040"/>
+            <a:ext cx="1866900" cy="739140"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
           <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="95000"/>
             </a:schemeClr>
           </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:fld id="{CAE52DA5-E783-42D2-873D-9F631120CFC5}" type="TxLink">
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="r"/>
+            <a:fld id="{CAE52DA5-E783-42D2-873D-9F631120CFC5}" type="TxLink">
+              <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mj-lt"/>
+              </a:rPr>
+              <a:pPr algn="r"/>
+              <a:t>31</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:latin typeface="+mj-lt"/>
-            </a:rPr>
-            <a:pPr algn="r"/>
-            <a:t>40</a:t>
-          </a:fld>
-          <a:endParaRPr lang="en-US" sz="2000" b="1">
-            <a:latin typeface="+mj-lt"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="8" name="Graphic 7" descr="Bar chart with solid fill">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D3243E3-E0D5-78A8-0AF9-066946EF9BEF}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+            <a:extLst>
+              <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5242560" y="845820"/>
+            <a:ext cx="457200" cy="457200"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>18358</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>141663</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="'data analysis'!E7">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="TextBox 3">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="14" name="Group 13">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9CF5D85A-1B58-1E0F-6ECB-D976385F9B60}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3285620-29D6-1D96-4D9D-BAAF38A9912E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7848600" y="701040"/>
-          <a:ext cx="1866900" cy="739140"/>
+          <a:off x="7901940" y="1664278"/>
+          <a:ext cx="1866900" cy="671945"/>
+          <a:chOff x="7848600" y="734638"/>
+          <a:chExt cx="1866900" cy="671945"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="'data analysis'!E7">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="4" name="TextBox 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9CF5D85A-1B58-1E0F-6ECB-D976385F9B60}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="7848600" y="734638"/>
+            <a:ext cx="1866900" cy="671945"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
           <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="95000"/>
             </a:schemeClr>
           </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:fld id="{5705C105-A208-49EE-830A-EA84537AE66E}" type="TxLink">
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Aptos Narrow"/>
-            </a:rPr>
-            <a:t>10663.25</a:t>
-          </a:fld>
-          <a:endParaRPr lang="en-US" sz="2000" b="1">
-            <a:latin typeface="Gotham" panose="02000504020000020004" pitchFamily="2" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="r"/>
+            <a:fld id="{5705C105-A208-49EE-830A-EA84537AE66E}" type="TxLink">
+              <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Aptos Narrow"/>
+              </a:rPr>
+              <a:t>9361</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-US" sz="2000" b="1">
+              <a:latin typeface="Gotham" panose="02000504020000020004" pitchFamily="2" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="10" name="Graphic 9" descr="Coins with solid fill">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{820BEEF1-CD67-BB33-C74D-0C2F9D4BEFEB}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+            <a:extLst>
+              <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="7947660" y="838200"/>
+            <a:ext cx="457200" cy="457200"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>601980</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>541020</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Graphic 5" descr="Money with solid fill">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAD87EE3-6A2A-DAE4-1F6A-4CBB4C810A49}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2522220" y="838200"/>
-          <a:ext cx="457200" cy="457200"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="11" name="Date 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48BEA061-2CC9-40DD-9566-8F872D9BD8FD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2012/timeslicer">
+              <tsle:timeslicer xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" name="Date 1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2430780" y="144780"/>
+              <a:ext cx="7322820" cy="1196340"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>Timeline: Works in Excel 2013 or higher. Do not move or resize.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>365760</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>213360</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>472440</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Graphic 7" descr="Bar chart with solid fill">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D3243E3-E0D5-78A8-0AF9-066946EF9BEF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5242560" y="845820"/>
-          <a:ext cx="457200" cy="457200"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>68580</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>525780</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Graphic 9" descr="Coins with solid fill">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{820BEEF1-CD67-BB33-C74D-0C2F9D4BEFEB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7993380" y="838200"/>
-          <a:ext cx="457200" cy="457200"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="3" name="Date">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{712F1F2D-AA36-429E-889B-E6B299DD56A9}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2012/timeslicer">
+              <tsle:timeslicer xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" name="Date"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4663440" y="937260"/>
+              <a:ext cx="3337560" cy="1181100"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>Timeline: Works in Excel 2013 or higher. Do not move or resize.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1568,13 +2263,13 @@
     <dataField name="AVG SALES" fld="7" subtotal="average" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="36">
+    <format dxfId="112">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="40" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="188" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -1712,13 +2407,13 @@
     <dataField name="TOTAL ITEM" fld="4" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="40">
+    <format dxfId="113">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="33" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="181" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -1856,13 +2551,13 @@
     <dataField name="TOTAL SALES" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="41">
+    <format dxfId="114">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="33" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="181" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -1911,10 +2606,10 @@
   <autoFilter ref="A1:H41" xr:uid="{DAE5D27C-AE6B-4686-951B-ABFA64A7EEE3}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{60EE4400-F973-4F15-948A-9008563AA622}" uniqueName="1" name="S No" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{A8629C8B-F662-4D64-94C6-C7B97196A735}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{5C50CE82-4D1A-4C79-9D0F-247FE1CDFA5C}" uniqueName="3" name="Salesman" queryTableFieldId="3" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{C594ECD2-D104-43F4-A766-C80694137000}" uniqueName="4" name="Region" queryTableFieldId="4" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{4EBFE9AF-2CF8-4086-910A-E4FE148003F0}" uniqueName="5" name="Item" queryTableFieldId="5" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{A8629C8B-F662-4D64-94C6-C7B97196A735}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="118"/>
+    <tableColumn id="3" xr3:uid="{5C50CE82-4D1A-4C79-9D0F-247FE1CDFA5C}" uniqueName="3" name="Salesman" queryTableFieldId="3" dataDxfId="117"/>
+    <tableColumn id="4" xr3:uid="{C594ECD2-D104-43F4-A766-C80694137000}" uniqueName="4" name="Region" queryTableFieldId="4" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{4EBFE9AF-2CF8-4086-910A-E4FE148003F0}" uniqueName="5" name="Item" queryTableFieldId="5" dataDxfId="115"/>
     <tableColumn id="6" xr3:uid="{28BA1440-E926-4945-883F-D0FCD7D3BB97}" uniqueName="6" name="Qty" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{9D812FB1-FCA4-4EB2-8FA6-297FD68B5A88}" uniqueName="7" name="Price" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{076B1DB5-2FB3-4FA7-8121-F2E26FB13E54}" uniqueName="8" name="Amount" queryTableFieldId="8"/>
@@ -2238,6 +2933,32 @@
 </a:theme>
 </file>
 
+<file path=xl/timelineCaches/timelineCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<timelineCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="xr10" name="NativeTimeline_Date" xr10:uid="{1A08CDD6-FD3D-453E-AB64-7E0795993188}" sourceName="Date">
+  <pivotTables>
+    <pivotTable tabId="3" name="PivotTable2"/>
+    <pivotTable tabId="3" name="PivotTable1"/>
+    <pivotTable tabId="3" name="PivotTable3"/>
+  </pivotTables>
+  <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="548194542" filterType="dateBetween">
+    <selection startDate="2023-01-01T00:00:00" endDate="2023-01-31T00:00:00"/>
+    <bounds startDate="2023-01-01T00:00:00" endDate="2024-01-01T00:00:00"/>
+  </state>
+</timelineCacheDefinition>
+</file>
+
+<file path=xl/timelines/timeline1.xml><?xml version="1.0" encoding="utf-8"?>
+<timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <timeline name="Date 1" xr10:uid="{4BAC2FE9-C0D7-4F7A-AA2C-A32B2D77E7A4}" cache="NativeTimeline_Date" caption="Date" showHorizontalScrollbar="0" level="2" selectionLevel="2" scrollPosition="2023-01-01T00:00:00" style="TimeSlicerStyleDark1"/>
+</timelines>
+</file>
+
+<file path=xl/timelines/timeline2.xml><?xml version="1.0" encoding="utf-8"?>
+<timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <timeline name="Date" xr10:uid="{8BE855AF-BCA8-4844-9C58-AD1748EA83F3}" cache="NativeTimeline_Date" caption="Date" showHorizontalScrollbar="0" level="2" selectionLevel="2" scrollPosition="2023-01-01T00:00:00"/>
+</timelines>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DC7FC4E-8D9E-4A1E-BCC5-B9D37254EE36}">
   <dimension ref="A1"/>
@@ -2245,6 +2966,13 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{7E03D99C-DC04-49d9-9315-930204A7B6E9}">
+      <x15:timelineRefs>
+        <x15:timelineRef r:id="rId2"/>
+      </x15:timelineRefs>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -2253,10 +2981,10 @@
   <dimension ref="A2:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2281,26 +3009,27 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
-        <v>426530</v>
+        <v>290180</v>
       </c>
       <c r="C6" s="4">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E6" s="4">
-        <v>10663.25</v>
+        <v>9360.645161290322</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
-        <v>426530</v>
+        <f>GETPIVOTDATA("Amount",$A$5)</f>
+        <v>290180</v>
       </c>
       <c r="C7">
         <f>GETPIVOTDATA("Item",$C$5)</f>
-        <v>40</v>
-      </c>
-      <c r="E7">
+        <v>31</v>
+      </c>
+      <c r="E7" s="7">
         <f>GETPIVOTDATA("Amount",$E$5)</f>
-        <v>10663.25</v>
+        <v>9360.645161290322</v>
       </c>
     </row>
   </sheetData>
@@ -2308,6 +3037,14 @@
     <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId4"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{7E03D99C-DC04-49d9-9315-930204A7B6E9}">
+      <x15:timelineRefs>
+        <x15:timelineRef r:id="rId5"/>
+      </x15:timelineRefs>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
dart update l file
</commit_message>
<xml_diff>
--- a/0B5F9D00.xlsx
+++ b/0B5F9D00.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\power bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84242AE8-80D1-469E-B6CB-B148ADC83800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44081467-0A3B-4521-8BE0-3FBB810044A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30BFA6B8-A676-4931-80C6-DA6F72E44419}"/>
   </bookViews>
@@ -243,7 +243,77 @@
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="142">
+  <dxfs count="152">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2065,7 +2135,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{8F04FACA-BB3F-456F-978F-18AE092E4DB8}" type="CELLRANGE">
+                <a:fld id="{D513CBE0-E094-4C26-96DA-DB434CB46CB4}" type="CELLRANGE">
                   <a:rPr lang="en-US"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2076,7 +2146,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{6C4A9361-0318-4687-8174-06F0597D5D29}" type="PERCENTAGE">
+                <a:fld id="{72920183-DA88-4872-88F3-A9CECC31E244}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2171,7 +2241,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{E8EA7B26-7E78-4AC7-BBF5-D1085E5A7553}" type="CELLRANGE">
+                <a:fld id="{50B8A57B-9ECA-4A6B-9F76-D0604A308663}" type="CELLRANGE">
                   <a:rPr lang="en-US"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2182,7 +2252,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{5FFDEAF5-0A11-4A88-87D1-98907541AF9D}" type="PERCENTAGE">
+                <a:fld id="{D0E6F6D9-C13A-437F-BE53-C2E24046A817}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2277,7 +2347,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{089C05EC-B45A-4671-B50E-34574E5C55A6}" type="CELLRANGE">
+                <a:fld id="{B3701F17-3C06-487F-9634-982686149457}" type="CELLRANGE">
                   <a:rPr lang="en-US"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2288,7 +2358,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{50D51559-626D-4A36-BB8E-3999BA1A592C}" type="PERCENTAGE">
+                <a:fld id="{38602BB4-B684-45A1-A60C-0E81C4D44DB3}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2383,7 +2453,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{53B4288B-A224-48D5-A844-84B01B96274D}" type="CELLRANGE">
+                <a:fld id="{80DB1AD1-58C2-4FE5-A975-4AA7F66E591B}" type="CELLRANGE">
                   <a:rPr lang="en-US"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2394,7 +2464,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{FBF05BD7-46BE-452E-B85F-5AA2B1D5BC3C}" type="PERCENTAGE">
+                <a:fld id="{5FC59D29-5B66-45B3-A6DC-0B54DECF4553}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -2561,7 +2631,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8F04FACA-BB3F-456F-978F-18AE092E4DB8}" type="CELLRANGE">
+                    <a:fld id="{D513CBE0-E094-4C26-96DA-DB434CB46CB4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2570,7 +2640,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{6C4A9361-0318-4687-8174-06F0597D5D29}" type="PERCENTAGE">
+                    <a:fld id="{72920183-DA88-4872-88F3-A9CECC31E244}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -2608,7 +2678,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E8EA7B26-7E78-4AC7-BBF5-D1085E5A7553}" type="CELLRANGE">
+                    <a:fld id="{50B8A57B-9ECA-4A6B-9F76-D0604A308663}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2617,7 +2687,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{5FFDEAF5-0A11-4A88-87D1-98907541AF9D}" type="PERCENTAGE">
+                    <a:fld id="{D0E6F6D9-C13A-437F-BE53-C2E24046A817}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -2655,7 +2725,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{089C05EC-B45A-4671-B50E-34574E5C55A6}" type="CELLRANGE">
+                    <a:fld id="{B3701F17-3C06-487F-9634-982686149457}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2664,7 +2734,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{50D51559-626D-4A36-BB8E-3999BA1A592C}" type="PERCENTAGE">
+                    <a:fld id="{38602BB4-B684-45A1-A60C-0E81C4D44DB3}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -2702,7 +2772,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{53B4288B-A224-48D5-A844-84B01B96274D}" type="CELLRANGE">
+                    <a:fld id="{80DB1AD1-58C2-4FE5-A975-4AA7F66E591B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2711,7 +2781,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{FBF05BD7-46BE-452E-B85F-5AA2B1D5BC3C}" type="PERCENTAGE">
+                    <a:fld id="{5FC59D29-5B66-45B3-A6DC-0B54DECF4553}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -8079,7 +8149,7 @@
     <dataField name="Sum of Amount" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="41">
+    <format dxfId="66">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -8210,7 +8280,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="231" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="261" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -8753,7 +8823,7 @@
     <dataField name="Sum of Amount" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="53">
+    <format dxfId="78">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -8779,7 +8849,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="231" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="261" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -9309,13 +9379,13 @@
     <dataField name="AVG SALES" fld="7" subtotal="average" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="135">
+    <format dxfId="145">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="231" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="261" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -9845,13 +9915,13 @@
     <dataField name="TOTAL ITEM" fld="4" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="136">
+    <format dxfId="146">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="224" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="254" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -10381,13 +10451,13 @@
     <dataField name="TOTAL SALES" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="137">
+    <format dxfId="147">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="1" type="dateBetween" evalOrder="-1" id="224" name="Date">
+    <filter fld="1" type="dateBetween" evalOrder="-1" id="254" name="Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -10436,10 +10506,10 @@
   <autoFilter ref="A1:H41" xr:uid="{DAE5D27C-AE6B-4686-951B-ABFA64A7EEE3}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{60EE4400-F973-4F15-948A-9008563AA622}" uniqueName="1" name="S No" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{A8629C8B-F662-4D64-94C6-C7B97196A735}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="141"/>
-    <tableColumn id="3" xr3:uid="{5C50CE82-4D1A-4C79-9D0F-247FE1CDFA5C}" uniqueName="3" name="Salesman" queryTableFieldId="3" dataDxfId="140"/>
-    <tableColumn id="4" xr3:uid="{C594ECD2-D104-43F4-A766-C80694137000}" uniqueName="4" name="Region" queryTableFieldId="4" dataDxfId="139"/>
-    <tableColumn id="5" xr3:uid="{4EBFE9AF-2CF8-4086-910A-E4FE148003F0}" uniqueName="5" name="Item" queryTableFieldId="5" dataDxfId="138"/>
+    <tableColumn id="2" xr3:uid="{A8629C8B-F662-4D64-94C6-C7B97196A735}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="151"/>
+    <tableColumn id="3" xr3:uid="{5C50CE82-4D1A-4C79-9D0F-247FE1CDFA5C}" uniqueName="3" name="Salesman" queryTableFieldId="3" dataDxfId="150"/>
+    <tableColumn id="4" xr3:uid="{C594ECD2-D104-43F4-A766-C80694137000}" uniqueName="4" name="Region" queryTableFieldId="4" dataDxfId="149"/>
+    <tableColumn id="5" xr3:uid="{4EBFE9AF-2CF8-4086-910A-E4FE148003F0}" uniqueName="5" name="Item" queryTableFieldId="5" dataDxfId="148"/>
     <tableColumn id="6" xr3:uid="{28BA1440-E926-4945-883F-D0FCD7D3BB97}" uniqueName="6" name="Qty" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{9D812FB1-FCA4-4EB2-8FA6-297FD68B5A88}" uniqueName="7" name="Price" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{076B1DB5-2FB3-4FA7-8121-F2E26FB13E54}" uniqueName="8" name="Amount" queryTableFieldId="8"/>

</xml_diff>

<commit_message>
change kpis card with new look
</commit_message>
<xml_diff>
--- a/0B5F9D00.xlsx
+++ b/0B5F9D00.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\power bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28A4B093-34FC-4ED4-A4C5-A3B6E851FECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF1FAAF8-3877-4538-9C50-7D78229FE8CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30BFA6B8-A676-4931-80C6-DA6F72E44419}"/>
   </bookViews>
@@ -315,6 +315,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFDD71"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1311,7 +1316,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{358BDF7D-75EF-412E-A458-8EDCA1788404}" type="CELLRANGE">
+                <a:fld id="{DA4B05AC-683C-4A27-AD91-C23E5434802F}" type="CELLRANGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -1322,7 +1327,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{3777432D-6524-49AA-895C-4B78A5F60EBA}" type="PERCENTAGE">
+                <a:fld id="{D3EA0865-3403-45FA-BC51-85AB7CCD831A}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr/>
@@ -1552,7 +1557,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{358BDF7D-75EF-412E-A458-8EDCA1788404}" type="CELLRANGE">
+                    <a:fld id="{DA4B05AC-683C-4A27-AD91-C23E5434802F}" type="CELLRANGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1561,7 +1566,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{3777432D-6524-49AA-895C-4B78A5F60EBA}" type="PERCENTAGE">
+                    <a:fld id="{D3EA0865-3403-45FA-BC51-85AB7CCD831A}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -8907,9 +8912,7 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="95000"/>
-          </a:schemeClr>
+          <a:srgbClr val="FFDD71"/>
         </a:solidFill>
         <a:ln>
           <a:noFill/>
@@ -9012,18 +9015,53 @@
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="bg1">
-              <a:lumMod val="95000"/>
-            </a:schemeClr>
-          </a:solidFill>
+          <a:gradFill flip="none" rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:srgbClr val="FFC000">
+                  <a:shade val="30000"/>
+                  <a:satMod val="115000"/>
+                </a:srgbClr>
+              </a:gs>
+              <a:gs pos="50000">
+                <a:srgbClr val="FFC000">
+                  <a:shade val="67500"/>
+                  <a:satMod val="115000"/>
+                </a:srgbClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:srgbClr val="FFC000">
+                  <a:shade val="100000"/>
+                  <a:satMod val="115000"/>
+                </a:srgbClr>
+              </a:gs>
+            </a:gsLst>
+            <a:path path="circle">
+              <a:fillToRect t="100000" r="100000"/>
+            </a:path>
+            <a:tileRect l="-100000" b="-100000"/>
+          </a:gradFill>
           <a:ln w="9525" cmpd="sng">
-            <a:solidFill>
-              <a:schemeClr val="lt1">
-                <a:shade val="50000"/>
-              </a:schemeClr>
-            </a:solidFill>
+            <a:noFill/>
           </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="190500" dist="228600" dir="2700000" algn="ctr">
+              <a:srgbClr val="000000">
+                <a:alpha val="30000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="glow" dir="t">
+              <a:rot lat="0" lon="0" rev="4800000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d prstMaterial="matte">
+            <a:bevelT w="127000" h="63500"/>
+          </a:sp3d>
         </xdr:spPr>
         <xdr:style>
           <a:lnRef idx="0">
@@ -9149,18 +9187,53 @@
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="bg1">
-              <a:lumMod val="95000"/>
-            </a:schemeClr>
-          </a:solidFill>
+          <a:gradFill flip="none" rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:srgbClr val="FFC000">
+                  <a:shade val="30000"/>
+                  <a:satMod val="115000"/>
+                </a:srgbClr>
+              </a:gs>
+              <a:gs pos="50000">
+                <a:srgbClr val="FFC000">
+                  <a:shade val="67500"/>
+                  <a:satMod val="115000"/>
+                </a:srgbClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:srgbClr val="FFC000">
+                  <a:shade val="100000"/>
+                  <a:satMod val="115000"/>
+                </a:srgbClr>
+              </a:gs>
+            </a:gsLst>
+            <a:path path="circle">
+              <a:fillToRect t="100000" r="100000"/>
+            </a:path>
+            <a:tileRect l="-100000" b="-100000"/>
+          </a:gradFill>
           <a:ln w="9525" cmpd="sng">
-            <a:solidFill>
-              <a:schemeClr val="lt1">
-                <a:shade val="50000"/>
-              </a:schemeClr>
-            </a:solidFill>
+            <a:noFill/>
           </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="190500" dist="228600" dir="2700000" algn="ctr">
+              <a:srgbClr val="000000">
+                <a:alpha val="30000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="glow" dir="t">
+              <a:rot lat="0" lon="0" rev="4800000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d prstMaterial="matte">
+            <a:bevelT w="127000" h="63500"/>
+          </a:sp3d>
         </xdr:spPr>
         <xdr:style>
           <a:lnRef idx="0">

</xml_diff>

<commit_message>
update vertical bar chart
</commit_message>
<xml_diff>
--- a/0B5F9D00.xlsx
+++ b/0B5F9D00.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\power bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D7C777-E6C9-4753-BB22-FC455F0ADDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8812050A-AFF7-4739-B474-798EB2756D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30BFA6B8-A676-4931-80C6-DA6F72E44419}"/>
   </bookViews>
@@ -251,56 +251,7 @@
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="18">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -415,11 +366,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FFFFDC6D"/>
       <color rgb="FF8A6900"/>
-      <color rgb="FFEEB500"/>
       <color rgb="FFFFECAF"/>
       <color rgb="FFFFDD71"/>
+      <color rgb="FFFFDC6D"/>
+      <color rgb="FFEEB500"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1369,7 +1320,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{BCEFE3A1-5279-439B-9D5C-5592E783B872}" type="CELLRANGE">
+                <a:fld id="{118FE687-2819-4DEB-9592-D9C8920A626F}" type="CELLRANGE">
                   <a:rPr lang="en-US"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1386,7 +1337,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{BAABADB7-2A00-4493-AEDA-37DF95019FAB}" type="PERCENTAGE">
+                <a:fld id="{ED12DC64-9EEB-4A45-B501-D90E15867279}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1483,7 +1434,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{2A40DA4D-081C-4A75-AF48-49C192B11051}" type="CELLRANGE">
+                <a:fld id="{5CC88ED6-2779-4F12-9818-188E0200F678}" type="CELLRANGE">
                   <a:rPr lang="en-US"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1500,7 +1451,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{1A6EE693-C9CB-4490-8154-3CC7F77D7522}" type="PERCENTAGE">
+                <a:fld id="{D825C52C-4859-4239-A32D-D07C356C206A}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1597,7 +1548,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{2EFC26A8-C002-4AAC-BD46-0D9C3C635444}" type="CELLRANGE">
+                <a:fld id="{43EEB421-DE47-458C-A076-0842EEDD3B95}" type="CELLRANGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1614,7 +1565,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{D58548AA-FB53-4E30-BE6C-815DA5FF1F09}" type="PERCENTAGE">
+                <a:fld id="{487044D8-0337-4544-BEFF-722A6CA889E4}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1711,7 +1662,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:fld id="{99CAD3F5-42F6-4700-BDEA-8BA293C1002D}" type="CELLRANGE">
+                <a:fld id="{77C4E1E9-C328-4B52-8D54-C4B8F0C76EC5}" type="CELLRANGE">
                   <a:rPr lang="en-US"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1728,7 +1679,7 @@
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:t>, </a:t>
                 </a:r>
-                <a:fld id="{0E8D410E-0079-4500-BF15-00B60B057867}" type="PERCENTAGE">
+                <a:fld id="{C8E53578-0B89-4022-BC29-ED43C2A9BEB2}" type="PERCENTAGE">
                   <a:rPr lang="en-US" baseline="0"/>
                   <a:pPr>
                     <a:defRPr b="1">
@@ -1892,7 +1843,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BCEFE3A1-5279-439B-9D5C-5592E783B872}" type="CELLRANGE">
+                    <a:fld id="{118FE687-2819-4DEB-9592-D9C8920A626F}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1901,7 +1852,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{BAABADB7-2A00-4493-AEDA-37DF95019FAB}" type="PERCENTAGE">
+                    <a:fld id="{ED12DC64-9EEB-4A45-B501-D90E15867279}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -1939,7 +1890,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2A40DA4D-081C-4A75-AF48-49C192B11051}" type="CELLRANGE">
+                    <a:fld id="{5CC88ED6-2779-4F12-9818-188E0200F678}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1948,7 +1899,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{1A6EE693-C9CB-4490-8154-3CC7F77D7522}" type="PERCENTAGE">
+                    <a:fld id="{D825C52C-4859-4239-A32D-D07C356C206A}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -1986,7 +1937,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2EFC26A8-C002-4AAC-BD46-0D9C3C635444}" type="CELLRANGE">
+                    <a:fld id="{43EEB421-DE47-458C-A076-0842EEDD3B95}" type="CELLRANGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1995,7 +1946,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{D58548AA-FB53-4E30-BE6C-815DA5FF1F09}" type="PERCENTAGE">
+                    <a:fld id="{487044D8-0337-4544-BEFF-722A6CA889E4}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -2033,7 +1984,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{99CAD3F5-42F6-4700-BDEA-8BA293C1002D}" type="CELLRANGE">
+                    <a:fld id="{77C4E1E9-C328-4B52-8D54-C4B8F0C76EC5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -2042,7 +1993,7 @@
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:t>, </a:t>
                     </a:r>
-                    <a:fld id="{0E8D410E-0079-4500-BF15-00B60B057867}" type="PERCENTAGE">
+                    <a:fld id="{C8E53578-0B89-4022-BC29-ED43C2A9BEB2}" type="PERCENTAGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[PERCENTAGE]</a:t>
@@ -3013,9 +2964,8 @@
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="bg2">
+                    <a:lumMod val="10000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -3024,14 +2974,32 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" b="1"/>
+              <a:rPr lang="en-US" b="1">
+                <a:solidFill>
+                  <a:schemeClr val="bg2">
+                    <a:lumMod val="10000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:rPr>
               <a:t>top</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" b="1" baseline="0"/>
+              <a:rPr lang="en-US" b="1" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="bg2">
+                    <a:lumMod val="10000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:rPr>
               <a:t> salers</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" b="1"/>
+            <a:endParaRPr lang="en-US" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="10000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -3050,9 +3018,8 @@
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="10000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -3208,11 +3175,11 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
+                      <a:lumMod val="95000"/>
+                      <a:lumOff val="5000"/>
                     </a:schemeClr>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
@@ -3234,6 +3201,78 @@
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
           </c:extLst>
         </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FFDD71"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FFDD71"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FFECAF"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FFECAF"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="7"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="8A6900"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="8"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="8A6900"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
       </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
@@ -3266,6 +3305,120 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="8A6900"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-42EE-4921-8F4A-7E5156F8A379}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="8A6900"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-42EE-4921-8F4A-7E5156F8A379}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFECAF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-42EE-4921-8F4A-7E5156F8A379}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFECAF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-42EE-4921-8F4A-7E5156F8A379}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFDD71"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-42EE-4921-8F4A-7E5156F8A379}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFDD71"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000000-42EE-4921-8F4A-7E5156F8A379}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:dLbls>
             <c:spPr>
               <a:noFill/>
@@ -3281,11 +3434,11 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
+                        <a:lumMod val="95000"/>
+                        <a:lumOff val="5000"/>
                       </a:schemeClr>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
@@ -3409,11 +3562,11 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
+                <a:lumMod val="95000"/>
+                <a:lumOff val="5000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -3425,11 +3578,11 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                    <a:lumMod val="95000"/>
+                    <a:lumOff val="5000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -3482,9 +3635,32 @@
     <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:srgbClr val="FFC000">
+            <a:shade val="30000"/>
+            <a:satMod val="115000"/>
+          </a:srgbClr>
+        </a:gs>
+        <a:gs pos="50000">
+          <a:srgbClr val="FFC000">
+            <a:shade val="67500"/>
+            <a:satMod val="115000"/>
+          </a:srgbClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:srgbClr val="FFC000">
+            <a:shade val="100000"/>
+            <a:satMod val="115000"/>
+          </a:srgbClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect t="100000" r="100000"/>
+      </a:path>
+      <a:tileRect l="-100000" b="-100000"/>
+    </a:gradFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
@@ -3495,6 +3671,13 @@
       <a:round/>
     </a:ln>
     <a:effectLst/>
+    <a:scene3d>
+      <a:camera prst="orthographicFront"/>
+      <a:lightRig rig="threePt" dir="t"/>
+    </a:scene3d>
+    <a:sp3d prstMaterial="matte">
+      <a:bevelT w="127000" h="63500"/>
+    </a:sp3d>
   </c:spPr>
   <c:txPr>
     <a:bodyPr/>
@@ -12936,7 +13119,7 @@
     <dataField name="Sum of Amount" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="18">
+    <format dxfId="11">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -13510,7 +13693,7 @@
     <dataField name="AVG SALES" fld="7" subtotal="average" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="19">
+    <format dxfId="12">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -14064,7 +14247,7 @@
     <dataField name="TOTAL ITEM" fld="4" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="20">
+    <format dxfId="13">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -14641,11 +14824,11 @@
     <dataField name="Sum of Amount" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="21">
+    <format dxfId="14">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
-  <chartFormats count="5">
+  <chartFormats count="11">
     <chartFormat chart="3" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -14686,6 +14869,78 @@
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
             <x v="0"/>
           </reference>
         </references>
@@ -15265,7 +15520,7 @@
     <dataField name="Sum of Amount" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="22">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -15909,7 +16164,7 @@
     <dataField name="TOTAL SALES" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="23">
+    <format dxfId="16">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -16480,7 +16735,7 @@
     <dataField name="Sum of Amount" fld="7" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="24">
+    <format dxfId="17">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -16772,10 +17027,10 @@
   <autoFilter ref="A1:H41" xr:uid="{DAE5D27C-AE6B-4686-951B-ABFA64A7EEE3}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{60EE4400-F973-4F15-948A-9008563AA622}" uniqueName="1" name="S No" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{A8629C8B-F662-4D64-94C6-C7B97196A735}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{5C50CE82-4D1A-4C79-9D0F-247FE1CDFA5C}" uniqueName="3" name="Salesman" queryTableFieldId="3" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{C594ECD2-D104-43F4-A766-C80694137000}" uniqueName="4" name="Region" queryTableFieldId="4" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{4EBFE9AF-2CF8-4086-910A-E4FE148003F0}" uniqueName="5" name="Item" queryTableFieldId="5" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{A8629C8B-F662-4D64-94C6-C7B97196A735}" uniqueName="2" name="Date" queryTableFieldId="2" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{5C50CE82-4D1A-4C79-9D0F-247FE1CDFA5C}" uniqueName="3" name="Salesman" queryTableFieldId="3" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{C594ECD2-D104-43F4-A766-C80694137000}" uniqueName="4" name="Region" queryTableFieldId="4" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{4EBFE9AF-2CF8-4086-910A-E4FE148003F0}" uniqueName="5" name="Item" queryTableFieldId="5" dataDxfId="7"/>
     <tableColumn id="6" xr3:uid="{28BA1440-E926-4945-883F-D0FCD7D3BB97}" uniqueName="6" name="Qty" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{9D812FB1-FCA4-4EB2-8FA6-297FD68B5A88}" uniqueName="7" name="Price" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{076B1DB5-2FB3-4FA7-8121-F2E26FB13E54}" uniqueName="8" name="Amount" queryTableFieldId="8"/>

</xml_diff>